<commit_message>
docs(design): structure v2 knobs on the Bond Rules sheet (rings, fades, shape traits)
Rows 43-59: per-ring fade (1.0, 0.6, 0.4, 0.25, 0.15) and runes each seal
adds (3, then 2), and five shape traits (closed ring, great ring, spoke,
branch, balanced) with first-pass changes. Written through Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/runes-workbook.xlsx
+++ b/design/runes-workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\lifesteal-crawler\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10267EE-787D-47A1-A719-C9DF58AE4238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB45486B-5F9E-48CC-8F12-E9DA11BA250C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -332,7 +332,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2679" uniqueCount="1674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2711" uniqueCount="1704">
   <si>
     <t>Passage rune workbook</t>
   </si>
@@ -5354,6 +5354,96 @@
   </si>
   <si>
     <t>2026-10-22: Effect (game) filled for all 166 base runes (the new affinities from their skill drafts), eleven runes revised after the modifier cross-check (hover a changed cell for what it was and why), and every rune's Skills on it filled from design/data-drafts/skills (176 skills).</t>
+  </si>
+  <si>
+    <t>Structure v2: seals as concentric rings (Brent 2026-10-23; first-pass numbers)</t>
+  </si>
+  <si>
+    <t>Each vestige binding forms a seal: a new ring around the skill. Forming a seal you may rework every inner ring and add the new one. Runes on a ring bond to their neighbours on that ring and to runes on the rings just inside and outside. A rune's strength = its ring's fade x the product of every bond's transmission on its path to the skill (each bond's kind factor, read from the side further out). An ionic bond hands the weaker rune's whole effect to the stronger rune.</t>
+  </si>
+  <si>
+    <t>Ring (seal)</t>
+  </si>
+  <si>
+    <t>Runes it adds</t>
+  </si>
+  <si>
+    <t>1 (first binding)</t>
+  </si>
+  <si>
+    <t>5 or more</t>
+  </si>
+  <si>
+    <t>Ring 1 plus the skill's own rune keeps Brent's "level 0 holds 4"; each later seal adds 2 ("+2 per level").</t>
+  </si>
+  <si>
+    <t>Shape trait</t>
+  </si>
+  <si>
+    <t>Needs</t>
+  </si>
+  <si>
+    <t>Change</t>
+  </si>
+  <si>
+    <t>What it means</t>
+  </si>
+  <si>
+    <t>Closed ring</t>
+  </si>
+  <si>
+    <t>every rune on a ring bonded round it</t>
+  </si>
+  <si>
+    <t>duration x1.2 per closed ring</t>
+  </si>
+  <si>
+    <t>the word holds itself together: the skill lasts longer</t>
+  </si>
+  <si>
+    <t>Great ring</t>
+  </si>
+  <si>
+    <t>a closed ring of 5 or more</t>
+  </si>
+  <si>
+    <t>repeats once at 40%</t>
+  </si>
+  <si>
+    <t>it comes round again</t>
+  </si>
+  <si>
+    <t>Spoke</t>
+  </si>
+  <si>
+    <t>a chain from ring 1 out through 3 or more rings</t>
+  </si>
+  <si>
+    <t>reach x1.15 and speed x1.15 per ring past the second</t>
+  </si>
+  <si>
+    <t>the word reaches out</t>
+  </si>
+  <si>
+    <t>a rune with 3 or more bonds</t>
+  </si>
+  <si>
+    <t>reach (area) x1.15 per branch rune, up to 3</t>
+  </si>
+  <si>
+    <t>the effect spreads</t>
+  </si>
+  <si>
+    <t>Balanced</t>
+  </si>
+  <si>
+    <t>ring 1 full, every bond to the skill the same kind</t>
+  </si>
+  <si>
+    <t>the skill's own rune keeps all of its nature</t>
+  </si>
+  <si>
+    <t>the skill stays itself</t>
   </si>
 </sst>
 </file>
@@ -5741,6 +5831,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -5752,9 +5845,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10608,32 +10698,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>942</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>928</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -10693,7 +10783,7 @@
         <v>Lull</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>943</v>
       </c>
       <c r="J6" s="10"/>
@@ -10724,7 +10814,7 @@
         <v>Blow</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1550</v>
       </c>
       <c r="J7" s="10"/>
@@ -10755,7 +10845,7 @@
         <v>Buffer</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1551</v>
       </c>
       <c r="J8" s="10"/>
@@ -10786,7 +10876,7 @@
         <v>Lash</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>947</v>
       </c>
       <c r="J9" s="10"/>
@@ -10817,7 +10907,7 @@
         <v>Drop</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>225</v>
       </c>
       <c r="J10" s="10"/>
@@ -10848,7 +10938,7 @@
         <v>Lift</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>229</v>
       </c>
       <c r="J11" s="10"/>
@@ -10879,7 +10969,7 @@
         <v>Stall</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1552</v>
       </c>
       <c r="J12" s="10"/>
@@ -10910,7 +11000,7 @@
         <v>Carry</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1553</v>
       </c>
       <c r="J13" s="10"/>
@@ -10941,7 +11031,7 @@
         <v>Disperse</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1554</v>
       </c>
       <c r="J14" s="10"/>
@@ -10972,7 +11062,7 @@
         <v>Whirl</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1555</v>
       </c>
       <c r="J15" s="10"/>
@@ -11015,32 +11105,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>950</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>928</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -11100,7 +11190,7 @@
         <v>Ground</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1556</v>
       </c>
       <c r="J6" s="10"/>
@@ -11131,7 +11221,7 @@
         <v>Strike</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>955</v>
       </c>
       <c r="J7" s="10"/>
@@ -11162,7 +11252,7 @@
         <v>Discharge</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>952</v>
       </c>
       <c r="J8" s="10"/>
@@ -11193,7 +11283,7 @@
         <v>Charge</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1210</v>
       </c>
       <c r="J9" s="10"/>
@@ -11224,7 +11314,7 @@
         <v>Insulate</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1557</v>
       </c>
       <c r="J10" s="10"/>
@@ -11255,7 +11345,7 @@
         <v>Arc</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1558</v>
       </c>
       <c r="J11" s="10"/>
@@ -11286,7 +11376,7 @@
         <v>Stun</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1559</v>
       </c>
       <c r="J12" s="10"/>
@@ -11317,7 +11407,7 @@
         <v>Quicken</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1560</v>
       </c>
       <c r="J13" s="10"/>
@@ -11348,7 +11438,7 @@
         <v>Silence</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1561</v>
       </c>
       <c r="J14" s="10"/>
@@ -11379,7 +11469,7 @@
         <v>Thunder</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1562</v>
       </c>
       <c r="J15" s="10"/>
@@ -11422,32 +11512,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>958</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>959</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -11505,7 +11595,7 @@
         <v>Thaw</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1563</v>
       </c>
       <c r="J6" s="10"/>
@@ -11534,7 +11624,7 @@
         <v>Freeze</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1564</v>
       </c>
       <c r="J7" s="10"/>
@@ -11563,7 +11653,7 @@
         <v>Glaze</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1565</v>
       </c>
       <c r="J8" s="10"/>
@@ -11592,7 +11682,7 @@
         <v>Frost</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1566</v>
       </c>
       <c r="J9" s="10"/>
@@ -11621,7 +11711,7 @@
         <v>Melt</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1567</v>
       </c>
       <c r="J10" s="10"/>
@@ -11650,7 +11740,7 @@
         <v>Snow</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1568</v>
       </c>
       <c r="J11" s="10"/>
@@ -11679,7 +11769,7 @@
         <v>Shatter</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1569</v>
       </c>
       <c r="J12" s="10"/>
@@ -11708,7 +11798,7 @@
         <v>Rime</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1570</v>
       </c>
       <c r="J13" s="10"/>
@@ -11737,7 +11827,7 @@
         <v>Toughen</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1571</v>
       </c>
       <c r="J14" s="10"/>
@@ -11766,7 +11856,7 @@
         <v>Brittle</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1572</v>
       </c>
       <c r="J15" s="10"/>
@@ -11809,32 +11899,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>966</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>967</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -11892,7 +11982,7 @@
         <v>Lighten</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1573</v>
       </c>
       <c r="J6" s="10"/>
@@ -11921,7 +12011,7 @@
         <v>Darken</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1574</v>
       </c>
       <c r="J7" s="10"/>
@@ -11950,7 +12040,7 @@
         <v>Expose</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1575</v>
       </c>
       <c r="J8" s="10"/>
@@ -11979,7 +12069,7 @@
         <v>Obscure</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1576</v>
       </c>
       <c r="J9" s="10"/>
@@ -12008,7 +12098,7 @@
         <v>Pin</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1577</v>
       </c>
       <c r="J10" s="10"/>
@@ -12037,7 +12127,7 @@
         <v>Shadowstep</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1578</v>
       </c>
       <c r="J11" s="10"/>
@@ -12066,7 +12156,7 @@
         <v>Resound</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1579</v>
       </c>
       <c r="J12" s="10"/>
@@ -12095,7 +12185,7 @@
         <v>Hush</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1580</v>
       </c>
       <c r="J13" s="10"/>
@@ -12124,7 +12214,7 @@
         <v>Disgorge</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1581</v>
       </c>
       <c r="J14" s="10"/>
@@ -12153,7 +12243,7 @@
         <v>Devour</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1582</v>
       </c>
       <c r="J15" s="10"/>
@@ -12196,32 +12286,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>974</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>975</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -12279,7 +12369,7 @@
         <v>Rust</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1583</v>
       </c>
       <c r="J6" s="10"/>
@@ -12308,7 +12398,7 @@
         <v>Forge</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1584</v>
       </c>
       <c r="J7" s="10"/>
@@ -12337,7 +12427,7 @@
         <v>Sunder</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1585</v>
       </c>
       <c r="J8" s="10"/>
@@ -12366,7 +12456,7 @@
         <v>Fuse</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1586</v>
       </c>
       <c r="J9" s="10"/>
@@ -12395,7 +12485,7 @@
         <v>Breach</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1587</v>
       </c>
       <c r="J10" s="10"/>
@@ -12424,7 +12514,7 @@
         <v>Seal</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1588</v>
       </c>
       <c r="J11" s="10"/>
@@ -12453,7 +12543,7 @@
         <v>Dull</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1589</v>
       </c>
       <c r="J12" s="10"/>
@@ -12482,7 +12572,7 @@
         <v>Hone</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1590</v>
       </c>
       <c r="J13" s="10"/>
@@ -12511,7 +12601,7 @@
         <v>Strip</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1591</v>
       </c>
       <c r="J14" s="10"/>
@@ -12540,7 +12630,7 @@
         <v>Plate</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1592</v>
       </c>
       <c r="J15" s="10"/>
@@ -12583,32 +12673,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>982</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>983</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -12666,7 +12756,7 @@
         <v>Staunch</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1593</v>
       </c>
       <c r="J6" s="10"/>
@@ -12695,7 +12785,7 @@
         <v>Bleed</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1594</v>
       </c>
       <c r="J7" s="10"/>
@@ -12724,7 +12814,7 @@
         <v>Spill</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1595</v>
       </c>
       <c r="J8" s="10"/>
@@ -12753,7 +12843,7 @@
         <v>Drink</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1596</v>
       </c>
       <c r="J9" s="10"/>
@@ -12782,7 +12872,7 @@
         <v>Thin</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1597</v>
       </c>
       <c r="J10" s="10"/>
@@ -12811,7 +12901,7 @@
         <v>Clot</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1598</v>
       </c>
       <c r="J11" s="10"/>
@@ -12840,7 +12930,7 @@
         <v>Still</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1599</v>
       </c>
       <c r="J12" s="10"/>
@@ -12869,7 +12959,7 @@
         <v>Pulse</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1600</v>
       </c>
       <c r="J13" s="10"/>
@@ -12898,7 +12988,7 @@
         <v>Breathe</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1601</v>
       </c>
       <c r="J14" s="10"/>
@@ -12927,7 +13017,7 @@
         <v>Choke</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1602</v>
       </c>
       <c r="J15" s="10"/>
@@ -12970,32 +13060,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>990</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>991</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -13053,7 +13143,7 @@
         <v>Wither</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1603</v>
       </c>
       <c r="J6" s="10"/>
@@ -13082,7 +13172,7 @@
         <v>Heal</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1604</v>
       </c>
       <c r="J7" s="10"/>
@@ -13111,7 +13201,7 @@
         <v>Exhaust</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1605</v>
       </c>
       <c r="J8" s="10"/>
@@ -13140,7 +13230,7 @@
         <v>Renew</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1606</v>
       </c>
       <c r="J9" s="10"/>
@@ -13169,7 +13259,7 @@
         <v>Weaken</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1607</v>
       </c>
       <c r="J10" s="10"/>
@@ -13198,7 +13288,7 @@
         <v>Strengthen</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1608</v>
       </c>
       <c r="J11" s="10"/>
@@ -13227,7 +13317,7 @@
         <v>Sicken</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1609</v>
       </c>
       <c r="J12" s="10"/>
@@ -13256,7 +13346,7 @@
         <v>Cure</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1610</v>
       </c>
       <c r="J13" s="10"/>
@@ -13285,7 +13375,7 @@
         <v>Arrest</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1611</v>
       </c>
       <c r="J14" s="10"/>
@@ -13314,7 +13404,7 @@
         <v>Regrow</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1612</v>
       </c>
       <c r="J15" s="10"/>
@@ -13357,32 +13447,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>996</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -13440,7 +13530,7 @@
         <v>Spare</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1613</v>
       </c>
       <c r="J6" s="10"/>
@@ -13469,7 +13559,7 @@
         <v>Kill</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1614</v>
       </c>
       <c r="J7" s="10"/>
@@ -13498,7 +13588,7 @@
         <v>Lay</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1615</v>
       </c>
       <c r="J8" s="10"/>
@@ -13527,7 +13617,7 @@
         <v>Animate</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1616</v>
       </c>
       <c r="J9" s="10"/>
@@ -13556,7 +13646,7 @@
         <v>Preserve</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1617</v>
       </c>
       <c r="J10" s="10"/>
@@ -13585,7 +13675,7 @@
         <v>Rot</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1618</v>
       </c>
       <c r="J11" s="10"/>
@@ -13614,7 +13704,7 @@
         <v>Exorcise</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1619</v>
       </c>
       <c r="J12" s="10"/>
@@ -13643,7 +13733,7 @@
         <v>Haunt</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1620</v>
       </c>
       <c r="J13" s="10"/>
@@ -13672,7 +13762,7 @@
         <v>Manifest</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1621</v>
       </c>
       <c r="J14" s="10"/>
@@ -13701,7 +13791,7 @@
         <v>Vanish</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1622</v>
       </c>
       <c r="J15" s="10"/>
@@ -13744,32 +13834,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>1006</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>1007</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -13827,7 +13917,7 @@
         <v>Shrink</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1623</v>
       </c>
       <c r="J6" s="10"/>
@@ -13856,7 +13946,7 @@
         <v>Grow</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1624</v>
       </c>
       <c r="J7" s="10"/>
@@ -13885,7 +13975,7 @@
         <v>Wilt</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1625</v>
       </c>
       <c r="J8" s="10"/>
@@ -13914,7 +14004,7 @@
         <v>Sprout</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1626</v>
       </c>
       <c r="J9" s="10"/>
@@ -13943,7 +14033,7 @@
         <v>Blight</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1627</v>
       </c>
       <c r="J10" s="10"/>
@@ -13972,7 +14062,7 @@
         <v>Flourish</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1628</v>
       </c>
       <c r="J11" s="10"/>
@@ -14001,7 +14091,7 @@
         <v>Sow</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1629</v>
       </c>
       <c r="J12" s="10"/>
@@ -14030,7 +14120,7 @@
         <v>Harvest</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1630</v>
       </c>
       <c r="J13" s="10"/>
@@ -14059,7 +14149,7 @@
         <v>Unravel</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1631</v>
       </c>
       <c r="J14" s="10"/>
@@ -14088,7 +14178,7 @@
         <v>Tangle</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1632</v>
       </c>
       <c r="J15" s="10"/>
@@ -14131,32 +14221,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>1011</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>1012</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -14214,7 +14304,7 @@
         <v>Dim</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1633</v>
       </c>
       <c r="J6" s="10"/>
@@ -14243,7 +14333,7 @@
         <v>Shine</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1634</v>
       </c>
       <c r="J7" s="10"/>
@@ -14272,7 +14362,7 @@
         <v>Glow</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1635</v>
       </c>
       <c r="J8" s="10"/>
@@ -14301,7 +14391,7 @@
         <v>Flash</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1636</v>
       </c>
       <c r="J9" s="10"/>
@@ -14330,7 +14420,7 @@
         <v>Absorb</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1637</v>
       </c>
       <c r="J10" s="10"/>
@@ -14359,7 +14449,7 @@
         <v>Radiate</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1638</v>
       </c>
       <c r="J11" s="10"/>
@@ -14388,7 +14478,7 @@
         <v>Clarity</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1639</v>
       </c>
       <c r="J12" s="10"/>
@@ -14417,7 +14507,7 @@
         <v>Glare</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1640</v>
       </c>
       <c r="J13" s="10"/>
@@ -14446,7 +14536,7 @@
         <v>Bend</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1641</v>
       </c>
       <c r="J14" s="10"/>
@@ -14475,7 +14565,7 @@
         <v>Reflect</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1642</v>
       </c>
       <c r="J15" s="10"/>
@@ -17177,32 +17267,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>1015</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>1016</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -17260,7 +17350,7 @@
         <v>Wake</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1643</v>
       </c>
       <c r="J6" s="10"/>
@@ -17289,7 +17379,7 @@
         <v>Sleep</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1644</v>
       </c>
       <c r="J7" s="10"/>
@@ -17318,7 +17408,7 @@
         <v>Dispel</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1645</v>
       </c>
       <c r="J8" s="10"/>
@@ -17347,7 +17437,7 @@
         <v>Conjure</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1646</v>
       </c>
       <c r="J9" s="10"/>
@@ -17376,7 +17466,7 @@
         <v>Soothe</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1647</v>
       </c>
       <c r="J10" s="10"/>
@@ -17405,7 +17495,7 @@
         <v>Dread</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1648</v>
       </c>
       <c r="J11" s="10"/>
@@ -17434,7 +17524,7 @@
         <v>Unmask</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1649</v>
       </c>
       <c r="J12" s="10"/>
@@ -17463,7 +17553,7 @@
         <v>Mimic</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1650</v>
       </c>
       <c r="J13" s="10"/>
@@ -17492,7 +17582,7 @@
         <v>Shut</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1651</v>
       </c>
       <c r="J14" s="10"/>
@@ -17521,7 +17611,7 @@
         <v>Whisper</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1652</v>
       </c>
       <c r="J15" s="10"/>
@@ -17564,32 +17654,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>1023</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>1012</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -17647,7 +17737,7 @@
         <v>Purge</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1653</v>
       </c>
       <c r="J6" s="10"/>
@@ -17676,7 +17766,7 @@
         <v>Poison</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1654</v>
       </c>
       <c r="J7" s="10"/>
@@ -17705,7 +17795,7 @@
         <v>Cleanse</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1655</v>
       </c>
       <c r="J8" s="10"/>
@@ -17734,7 +17824,7 @@
         <v>Contaminate</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1656</v>
       </c>
       <c r="J9" s="10"/>
@@ -17763,7 +17853,7 @@
         <v>Neutralise</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1657</v>
       </c>
       <c r="J10" s="10"/>
@@ -17792,7 +17882,7 @@
         <v>Corrode</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1658</v>
       </c>
       <c r="J11" s="10"/>
@@ -17821,7 +17911,7 @@
         <v>Flush</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1659</v>
       </c>
       <c r="J12" s="10"/>
@@ -17850,7 +17940,7 @@
         <v>Linger</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1660</v>
       </c>
       <c r="J13" s="10"/>
@@ -17879,7 +17969,7 @@
         <v>Stimulate</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1661</v>
       </c>
       <c r="J14" s="10"/>
@@ -17908,7 +17998,7 @@
         <v>Sap</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1662</v>
       </c>
       <c r="J15" s="10"/>
@@ -17951,32 +18041,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>1030</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>1031</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -18034,7 +18124,7 @@
         <v>Disinfect</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1663</v>
       </c>
       <c r="J6" s="10"/>
@@ -18063,7 +18153,7 @@
         <v>Infect</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1609</v>
       </c>
       <c r="J7" s="10"/>
@@ -18092,7 +18182,7 @@
         <v>Contain</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1664</v>
       </c>
       <c r="J8" s="10"/>
@@ -18121,7 +18211,7 @@
         <v>Spread</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1665</v>
       </c>
       <c r="J9" s="10"/>
@@ -18150,7 +18240,7 @@
         <v>Lance</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1666</v>
       </c>
       <c r="J10" s="10"/>
@@ -18179,7 +18269,7 @@
         <v>Fester</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1667</v>
       </c>
       <c r="J11" s="10"/>
@@ -18208,7 +18298,7 @@
         <v>Clear</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1668</v>
       </c>
       <c r="J12" s="10"/>
@@ -18237,7 +18327,7 @@
         <v>Billow</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1669</v>
       </c>
       <c r="J13" s="10"/>
@@ -18266,7 +18356,7 @@
         <v>Immunise</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1670</v>
       </c>
       <c r="J14" s="10"/>
@@ -18295,7 +18385,7 @@
         <v>Overrun</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1671</v>
       </c>
       <c r="J15" s="10"/>
@@ -30620,7 +30710,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{707B76BF-2512-40E2-935C-38AB239C315D}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="31" customWidth="1"/>
@@ -30730,13 +30820,13 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="60" t="s">
         <v>1081</v>
       </c>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="44" t="s">
@@ -30783,13 +30873,13 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="60" t="s">
+      <c r="A17" s="61" t="s">
         <v>1091</v>
       </c>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
     </row>
     <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="58" t="s">
@@ -30797,13 +30887,13 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="59" t="s">
+      <c r="A20" s="60" t="s">
         <v>1392</v>
       </c>
-      <c r="B20" s="59"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="59"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="60"/>
     </row>
     <row r="22" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A22" s="35" t="s">
@@ -30934,25 +31024,200 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="59" t="s">
+      <c r="A38" s="60" t="s">
         <v>1406</v>
       </c>
-      <c r="B38" s="59"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="59"/>
-      <c r="E38" s="59"/>
+      <c r="B38" s="60"/>
+      <c r="C38" s="60"/>
+      <c r="D38" s="60"/>
+      <c r="E38" s="60"/>
     </row>
     <row r="40" spans="1:5" ht="110.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="59" t="s">
+      <c r="A40" s="60" t="s">
         <v>1672</v>
       </c>
-      <c r="B40" s="59"/>
-      <c r="C40" s="59"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="59"/>
+      <c r="B40" s="60"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="60"/>
+      <c r="E40" s="60"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="58" t="s">
+        <v>1674</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="56.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="60" t="s">
+        <v>1675</v>
+      </c>
+      <c r="B44" s="60"/>
+      <c r="C44" s="60"/>
+      <c r="D44" s="60"/>
+      <c r="E44" s="60"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="35" t="s">
+        <v>1676</v>
+      </c>
+      <c r="B46" s="35" t="s">
+        <v>766</v>
+      </c>
+      <c r="C46" s="35" t="s">
+        <v>1677</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="40" t="s">
+        <v>1678</v>
+      </c>
+      <c r="B47" s="33">
+        <v>1</v>
+      </c>
+      <c r="C47" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="40">
+        <v>2</v>
+      </c>
+      <c r="B48" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="C48" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="40">
+        <v>3</v>
+      </c>
+      <c r="B49" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="C49" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="40">
+        <v>4</v>
+      </c>
+      <c r="B50" s="33">
+        <v>0.25</v>
+      </c>
+      <c r="C50" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="40" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B51" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="C51" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="60" t="s">
+        <v>1680</v>
+      </c>
+      <c r="B52" s="60"/>
+      <c r="C52" s="60"/>
+      <c r="D52" s="60"/>
+      <c r="E52" s="60"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="35" t="s">
+        <v>1681</v>
+      </c>
+      <c r="B54" s="35" t="s">
+        <v>1682</v>
+      </c>
+      <c r="C54" s="35" t="s">
+        <v>1683</v>
+      </c>
+      <c r="D54" s="35" t="s">
+        <v>1684</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A55" s="40" t="s">
+        <v>1685</v>
+      </c>
+      <c r="B55" s="40" t="s">
+        <v>1686</v>
+      </c>
+      <c r="C55" s="33" t="s">
+        <v>1687</v>
+      </c>
+      <c r="D55" s="40" t="s">
+        <v>1688</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A56" s="40" t="s">
+        <v>1689</v>
+      </c>
+      <c r="B56" s="40" t="s">
+        <v>1690</v>
+      </c>
+      <c r="C56" s="33" t="s">
+        <v>1691</v>
+      </c>
+      <c r="D56" s="40" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A57" s="40" t="s">
+        <v>1693</v>
+      </c>
+      <c r="B57" s="40" t="s">
+        <v>1694</v>
+      </c>
+      <c r="C57" s="33" t="s">
+        <v>1695</v>
+      </c>
+      <c r="D57" s="40" t="s">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A58" s="40" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B58" s="40" t="s">
+        <v>1697</v>
+      </c>
+      <c r="C58" s="33" t="s">
+        <v>1698</v>
+      </c>
+      <c r="D58" s="40" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A59" s="40" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B59" s="40" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C59" s="33" t="s">
+        <v>1702</v>
+      </c>
+      <c r="D59" s="40" t="s">
+        <v>1703</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A20:E20"/>
@@ -30987,32 +31252,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>903</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>904</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -31072,7 +31337,7 @@
         <v>Drain</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>917</v>
       </c>
       <c r="J6" s="10" t="s">
@@ -31105,7 +31370,7 @@
         <v>Flood</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1525</v>
       </c>
       <c r="J7" s="10"/>
@@ -31138,7 +31403,7 @@
       <c r="H8" s="10" t="s">
         <v>1173</v>
       </c>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>912</v>
       </c>
       <c r="J8" s="10"/>
@@ -31171,7 +31436,7 @@
       <c r="H9" s="10" t="s">
         <v>1173</v>
       </c>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>915</v>
       </c>
       <c r="J9" s="10"/>
@@ -31204,7 +31469,7 @@
       <c r="H10" s="10" t="s">
         <v>1174</v>
       </c>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1526</v>
       </c>
       <c r="J10" s="10"/>
@@ -31237,7 +31502,7 @@
       <c r="H11" s="10" t="s">
         <v>1174</v>
       </c>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>1527</v>
       </c>
       <c r="J11" s="10" t="s">
@@ -31272,7 +31537,7 @@
       <c r="H12" s="10" t="s">
         <v>1178</v>
       </c>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1528</v>
       </c>
       <c r="J12" s="10"/>
@@ -31305,7 +31570,7 @@
       <c r="H13" s="10" t="s">
         <v>1178</v>
       </c>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1529</v>
       </c>
       <c r="J13" s="10" t="s">
@@ -31338,7 +31603,7 @@
         <v>Drip</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>922</v>
       </c>
       <c r="J14" s="10"/>
@@ -31369,7 +31634,7 @@
         <v>Gush</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1530</v>
       </c>
       <c r="J15" s="10"/>
@@ -31400,7 +31665,7 @@
         <v>Settle</v>
       </c>
       <c r="H16" s="55"/>
-      <c r="I16" s="64" t="s">
+      <c r="I16" s="59" t="s">
         <v>916</v>
       </c>
       <c r="J16" s="10"/>
@@ -31431,7 +31696,7 @@
         <v>Sweep</v>
       </c>
       <c r="H17" s="55"/>
-      <c r="I17" s="64" t="s">
+      <c r="I17" s="59" t="s">
         <v>1531</v>
       </c>
       <c r="J17" s="10"/>
@@ -31462,7 +31727,7 @@
         <v>Seep</v>
       </c>
       <c r="H18" s="55"/>
-      <c r="I18" s="64" t="s">
+      <c r="I18" s="59" t="s">
         <v>924</v>
       </c>
       <c r="J18" s="10"/>
@@ -31493,7 +31758,7 @@
         <v>Splash</v>
       </c>
       <c r="H19" s="55"/>
-      <c r="I19" s="64" t="s">
+      <c r="I19" s="59" t="s">
         <v>1532</v>
       </c>
       <c r="J19" s="10"/>
@@ -31524,7 +31789,7 @@
         <v>Slack</v>
       </c>
       <c r="H20" s="55"/>
-      <c r="I20" s="64" t="s">
+      <c r="I20" s="59" t="s">
         <v>1533</v>
       </c>
       <c r="J20" s="10"/>
@@ -31555,7 +31820,7 @@
         <v>Wave</v>
       </c>
       <c r="H21" s="55"/>
-      <c r="I21" s="64" t="s">
+      <c r="I21" s="59" t="s">
         <v>1534</v>
       </c>
       <c r="J21" s="10"/>
@@ -31598,32 +31863,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>927</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>928</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -31683,7 +31948,7 @@
         <v>Quench</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1535</v>
       </c>
       <c r="J6" s="10"/>
@@ -31714,7 +31979,7 @@
         <v>Burn</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1536</v>
       </c>
       <c r="J7" s="10"/>
@@ -31745,7 +32010,7 @@
         <v>Snuff</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>1537</v>
       </c>
       <c r="J8" s="10"/>
@@ -31776,7 +32041,7 @@
         <v>Ignite</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1538</v>
       </c>
       <c r="J9" s="10"/>
@@ -31807,7 +32072,7 @@
         <v>Implode</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>1193</v>
       </c>
       <c r="J10" s="10"/>
@@ -31838,7 +32103,7 @@
         <v>Explode</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>931</v>
       </c>
       <c r="J11" s="10"/>
@@ -31869,7 +32134,7 @@
         <v>Smoulder</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1539</v>
       </c>
       <c r="J12" s="10"/>
@@ -31900,7 +32165,7 @@
         <v>Blaze</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1540</v>
       </c>
       <c r="J13" s="10"/>
@@ -31931,7 +32196,7 @@
         <v>Smother</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1541</v>
       </c>
       <c r="J14" s="10"/>
@@ -31962,7 +32227,7 @@
         <v>Flare</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1542</v>
       </c>
       <c r="J15" s="10"/>
@@ -32005,32 +32270,32 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>932</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="62" t="s">
         <v>928</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -32090,7 +32355,7 @@
         <v>Sink</v>
       </c>
       <c r="H6" s="55"/>
-      <c r="I6" s="64" t="s">
+      <c r="I6" s="59" t="s">
         <v>1543</v>
       </c>
       <c r="J6" s="10"/>
@@ -32121,7 +32386,7 @@
         <v>Raise</v>
       </c>
       <c r="H7" s="55"/>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="59" t="s">
         <v>1544</v>
       </c>
       <c r="J7" s="10"/>
@@ -32152,7 +32417,7 @@
         <v>Crumble</v>
       </c>
       <c r="H8" s="55"/>
-      <c r="I8" s="64" t="s">
+      <c r="I8" s="59" t="s">
         <v>936</v>
       </c>
       <c r="J8" s="10"/>
@@ -32183,7 +32448,7 @@
         <v>Harden</v>
       </c>
       <c r="H9" s="55"/>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="59" t="s">
         <v>1545</v>
       </c>
       <c r="J9" s="10"/>
@@ -32214,7 +32479,7 @@
         <v>Quake</v>
       </c>
       <c r="H10" s="55"/>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="59" t="s">
         <v>939</v>
       </c>
       <c r="J10" s="10"/>
@@ -32245,7 +32510,7 @@
         <v>Root</v>
       </c>
       <c r="H11" s="55"/>
-      <c r="I11" s="64" t="s">
+      <c r="I11" s="59" t="s">
         <v>941</v>
       </c>
       <c r="J11" s="10"/>
@@ -32276,7 +32541,7 @@
         <v>Bury</v>
       </c>
       <c r="H12" s="55"/>
-      <c r="I12" s="64" t="s">
+      <c r="I12" s="59" t="s">
         <v>1546</v>
       </c>
       <c r="J12" s="10"/>
@@ -32307,7 +32572,7 @@
         <v>Dig</v>
       </c>
       <c r="H13" s="55"/>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="59" t="s">
         <v>1547</v>
       </c>
       <c r="J13" s="10"/>
@@ -32338,7 +32603,7 @@
         <v>Collapse</v>
       </c>
       <c r="H14" s="55"/>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="59" t="s">
         <v>1548</v>
       </c>
       <c r="J14" s="10"/>
@@ -32369,7 +32634,7 @@
         <v>Tunnel</v>
       </c>
       <c r="H15" s="55"/>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="59" t="s">
         <v>1549</v>
       </c>
       <c r="J15" s="10"/>

</xml_diff>

<commit_message>
docs(design): strength on on/off effects and ionic conversion knobs (Bond Rules rows 62-74)
Brent 2026-10-23: dominance must pay. Statuses and interrupts grow with
strength (longer, deeper, interrupt becomes silence) and an ionic bond
converts what the weaker side gives up into the stronger rune's strength.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/runes-workbook.xlsx
+++ b/design/runes-workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\lifesteal-crawler\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB45486B-5F9E-48CC-8F12-E9DA11BA250C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD8F037-8EBA-4471-AF20-5E9B3D76011B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -332,7 +332,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2711" uniqueCount="1704">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2731" uniqueCount="1723">
   <si>
     <t>Passage rune workbook</t>
   </si>
@@ -5444,6 +5444,63 @@
   </si>
   <si>
     <t>the skill stays itself</t>
+  </si>
+  <si>
+    <t>Strength on on/off effects, and ionic conversion (Brent 2026-10-23; first-pass numbers)</t>
+  </si>
+  <si>
+    <t>Dominance must pay: an on/off effect (a status, an interrupt) also grows with strength, and in an ionic bond nothing is lost - what the weaker side gives up is converted into the stronger rune's strength.</t>
+  </si>
+  <si>
+    <t>Knob</t>
+  </si>
+  <si>
+    <t>What it does</t>
+  </si>
+  <si>
+    <t>Status duration per strength</t>
+  </si>
+  <si>
+    <t>a status lasts base x strength (above 1 it lasts longer)</t>
+  </si>
+  <si>
+    <t>Status duration cap</t>
+  </si>
+  <si>
+    <t>longest a status can be stretched, as a multiple of its base</t>
+  </si>
+  <si>
+    <t>Extra stack per strength above 1</t>
+  </si>
+  <si>
+    <t>each full 1.0 of strength above 1 adds a stack (where the status stacks)</t>
+  </si>
+  <si>
+    <t>Interrupt becomes silence above strength</t>
+  </si>
+  <si>
+    <t>an interrupt at higher strength also stops casting</t>
+  </si>
+  <si>
+    <t>Silence seconds per strength above 1</t>
+  </si>
+  <si>
+    <t>how long the silence lasts per 1.0 of strength above the line</t>
+  </si>
+  <si>
+    <t>Ionic conversion rate</t>
+  </si>
+  <si>
+    <t>share of what the weaker side gives up that is added to the stronger rune's strength</t>
+  </si>
+  <si>
+    <t>Converted strength cap</t>
+  </si>
+  <si>
+    <t>the most strength a rune can reach by conversion</t>
+  </si>
+  <si>
+    <t>Example: Drown takes Wave (ionic) on Tidal Bore. Wave gives up all of its nature (reach, stagger, carry), so Drown's strength goes 1.5 -&gt; 2.5: its interrupt becomes a 2.25 s silence and Dazed lasts 2.5x as long.</t>
   </si>
 </sst>
 </file>
@@ -30710,7 +30767,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{707B76BF-2512-40E2-935C-38AB239C315D}">
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="31" customWidth="1"/>
@@ -31214,8 +31271,121 @@
         <v>1703</v>
       </c>
     </row>
+    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="58" t="s">
+        <v>1704</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="60" t="s">
+        <v>1705</v>
+      </c>
+      <c r="B63" s="60"/>
+      <c r="C63" s="60"/>
+      <c r="D63" s="60"/>
+      <c r="E63" s="60"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" s="35" t="s">
+        <v>1706</v>
+      </c>
+      <c r="B65" s="35" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C65" s="35" t="s">
+        <v>1707</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A66" s="40" t="s">
+        <v>1708</v>
+      </c>
+      <c r="B66" s="33">
+        <v>1</v>
+      </c>
+      <c r="C66" s="40" t="s">
+        <v>1709</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A67" s="40" t="s">
+        <v>1710</v>
+      </c>
+      <c r="B67" s="33">
+        <v>2.5</v>
+      </c>
+      <c r="C67" s="40" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A68" s="40" t="s">
+        <v>1712</v>
+      </c>
+      <c r="B68" s="33">
+        <v>1</v>
+      </c>
+      <c r="C68" s="40" t="s">
+        <v>1713</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A69" s="40" t="s">
+        <v>1714</v>
+      </c>
+      <c r="B69" s="33">
+        <v>1</v>
+      </c>
+      <c r="C69" s="40" t="s">
+        <v>1715</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A70" s="40" t="s">
+        <v>1716</v>
+      </c>
+      <c r="B70" s="33">
+        <v>1.5</v>
+      </c>
+      <c r="C70" s="40" t="s">
+        <v>1717</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A71" s="40" t="s">
+        <v>1718</v>
+      </c>
+      <c r="B71" s="33">
+        <v>1</v>
+      </c>
+      <c r="C71" s="40" t="s">
+        <v>1719</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A72" s="40" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B72" s="33">
+        <v>3</v>
+      </c>
+      <c r="C72" s="40" t="s">
+        <v>1721</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="60" t="s">
+        <v>1722</v>
+      </c>
+      <c r="B74" s="60"/>
+      <c r="C74" s="60"/>
+      <c r="D74" s="60"/>
+      <c r="E74" s="60"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A74:E74"/>
     <mergeCell ref="A44:E44"/>
     <mergeCell ref="A52:E52"/>
     <mergeCell ref="A10:E10"/>

</xml_diff>